<commit_message>
Save point: Aula4[ semana 05, analise de dados
</commit_message>
<xml_diff>
--- a/Analise_de_dados_e_IA_Nivelamento/Semana_05/Analise_de_dados_Calculos_padroes_e_estrategias_com_Excel/03_Medidas_de_Dispersao/db/Base_dados.xlsx
+++ b/Analise_de_dados_e_IA_Nivelamento/Semana_05/Analise_de_dados_Calculos_padroes_e_estrategias_com_Excel/03_Medidas_de_Dispersao/db/Base_dados.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thierry-G15\Documents\Estudos\Alura\Santander-Imersao-Digital\Analise_de_dados_e_IA_Nivelamento\Semana_05\Analise_de_dados_Calculos_padroes_e_estrategias_com_Excel\02_Medidas_de_Posicao\db\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thierry-G15\Documents\Estudos\Alura\Santander-Imersao-Digital\Analise_de_dados_e_IA_Nivelamento\Semana_05\Analise_de_dados_Calculos_padroes_e_estrategias_com_Excel\03_Medidas_de_Dispersao\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7150FF1-CC2B-4452-BFC9-F234D97D662D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{854DAFC0-F227-4596-A8DE-23489857D3E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-4080" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{D7F695BB-FECC-43AA-BDAB-82D9C8DC47D6}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3071" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3075" uniqueCount="89">
   <si>
     <t>Home Office</t>
   </si>
@@ -299,6 +299,18 @@
   </si>
   <si>
     <t>Media de lucro para Corporativo</t>
+  </si>
+  <si>
+    <t>Média de Lucro</t>
+  </si>
+  <si>
+    <t>Desvio Médio</t>
+  </si>
+  <si>
+    <t>Variância</t>
+  </si>
+  <si>
+    <t>Desvio Padrão</t>
   </si>
 </sst>
 </file>
@@ -18973,6 +18985,9 @@
       <c r="M11">
         <v>50.8</v>
       </c>
+      <c r="N11" s="3" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -19014,6 +19029,10 @@
       <c r="M12">
         <v>49.68</v>
       </c>
+      <c r="N12">
+        <f>AVERAGE(M:M)</f>
+        <v>1.1446799999999868</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -19055,6 +19074,9 @@
       <c r="M13">
         <v>32.270000000000003</v>
       </c>
+      <c r="N13" s="3" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -19096,6 +19118,10 @@
       <c r="M14">
         <v>5.0599999999999996</v>
       </c>
+      <c r="N14">
+        <f>AVEDEV(M:M)</f>
+        <v>65.453736320000004</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -19137,6 +19163,9 @@
       <c r="M15">
         <v>20.45</v>
       </c>
+      <c r="N15" s="3" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -19178,8 +19207,12 @@
       <c r="M16">
         <v>21.35</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N16">
+        <f>_xlfn.VAR.S(M:M)</f>
+        <v>88033.598174847299</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -19219,8 +19252,11 @@
       <c r="M17">
         <v>3.93</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N17" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -19260,8 +19296,12 @@
       <c r="M18">
         <v>582.07000000000005</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N18">
+        <f>_xlfn.STDEV.S(M:M)</f>
+        <v>296.70456379174101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -19301,8 +19341,12 @@
       <c r="M19">
         <v>33.47</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N19">
+        <f>AVEDEV(K:K)</f>
+        <v>269.31249431999998</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -19343,7 +19387,7 @@
         <v>23.03</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -19384,7 +19428,7 @@
         <v>479.69</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -19425,7 +19469,7 @@
         <v>8.59</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -19466,7 +19510,7 @@
         <v>-7.33</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -19507,7 +19551,7 @@
         <v>3.09</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -19548,7 +19592,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -19589,7 +19633,7 @@
         <v>17.809999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -19630,7 +19674,7 @@
         <v>4628.04</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -19671,7 +19715,7 @@
         <v>10.53</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -19712,7 +19756,7 @@
         <v>72.91</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -19753,7 +19797,7 @@
         <v>16.11</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -19794,7 +19838,7 @@
         <v>53.15</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>

</xml_diff>